<commit_message>
replace team with howell -p 4
</commit_message>
<xml_diff>
--- a/howell5.xlsx
+++ b/howell5.xlsx
@@ -506,7 +506,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>For public domain. No rights reserved. Generated on Mar 20, 2026.</t>
+          <t>For public domain. No rights reserved. Generated on Apr 08, 2026.</t>
         </is>
       </c>
     </row>
@@ -590,12 +590,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Name 80</t>
+          <t>Name 29</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Name 83</t>
+          <t>Name 55</t>
         </is>
       </c>
       <c r="D10" s="4">
@@ -613,7 +613,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Name 46</t>
+          <t>Name 82</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -636,12 +636,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Name 56</t>
+          <t>Name 27</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Name 16</t>
+          <t>Name 25</t>
         </is>
       </c>
       <c r="D12" s="4">
@@ -659,12 +659,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Name 39</t>
+          <t>Name 23</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Name 44</t>
+          <t>Name 67</t>
         </is>
       </c>
       <c r="D13" s="4">
@@ -682,12 +682,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Name 86</t>
+          <t>Name 19</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Name 40</t>
+          <t>Name 34</t>
         </is>
       </c>
       <c r="D14" s="4">

</xml_diff>